<commit_message>
Track 2 v2 additions: NAD+ precursor grading and pseudokinase stabilizer screen
- NAD+ precursors graded against North 2014 with the ChEMBL coverage gap documented
  (niacin rejected for this case; nicotinamide direction-conflict; acipimox no FDA approval)
- Bounded stabilizer docking screen over 2,240 approved ligands against three BUBR1
  pseudokinase pockets: honest negative with declared instrument limit (ADP redock 6.03 A)
- Report v2, methods form v2 (regenerated), pitch outline v2, screen pipeline source
</commit_message>
<xml_diff>
--- a/track2/Silico-EVEE_track2_methods_description_form_v2.xlsx
+++ b/track2/Silico-EVEE_track2_methods_description_form_v2.xlsx
@@ -679,7 +679,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Two layered passes over the same verified mechanism chain. First layer (v1): the variant mechanism was rebuilt from public primary sources (Ensembl REST for the 23-exon MANE transcript ENST00000287598, UniProt O60566, AlphaFold DB AF-O60566-F1, ClinVar VCV000533901.9), and candidate classes were screened with fixed Europe PMC queries and graded on five axes (mechanism tie, preclinical evidence, regulator-verified status, pediatric labeling, tumor fit). Second layer (v2): a quantitative screen over the full approved-drug space, ChEMBL 37 max_phase=4 direct-interaction mechanisms (1,811 drugs, 650 human targets, 3,927 drug-gene rows), scored on three orthogonal lanes. Lane 1 network proximity: Guney z-scores against a pre-declared 12-gene MVA module over BioGRID 4.4.236 human physical PPI, 1,000 degree-matched nulls, seed 42 (calibrations: ivacaftor-CFTR z=-3.41, imatinib-BCR/ABL1 z=-10.66). Lane 2 knowledge graph: Bioteque disgenet-inferred bundle, cosine to the MVA1 node DOID:0080141 (self-edge AUC 0.917 calibration). Lane 3 signature reversal: BUB1B-knockdown proxy from GEO GSE92742 Phase I, 58 quality-gated signatures, tau-style connectivity over 205,034 compound signatures; the lane declares its own instrument limit (held-out-hairpin reconnection 0.101 vs null p95 0.184) and is used as weak evidence only. Structural allele tickets: RaSP stability scan on the AlphaFold model (N1002K ddG +2.41 kcal/mol in the validated I909T class; identity band +0.39 sd 0.58) and fpocket 4.2.3 (97 pockets, no druggable pocket at the locus). A pre-declared rule bans screen-score-only promotion; verdicts are graded on published direct evidence, regulator-verified status, and pediatric feasibility.</t>
+          <t>Two layered passes over the same verified mechanism chain. First layer (v1): the variant mechanism was rebuilt from public primary sources (Ensembl REST for the 23-exon MANE transcript ENST00000287598, UniProt O60566, AlphaFold DB AF-O60566-F1, ClinVar VCV000533901.9), and candidate classes were screened with fixed Europe PMC queries and graded on five axes (mechanism tie, preclinical evidence, regulator-verified status, pediatric labeling, tumor fit). Second layer (v2): a quantitative screen over the full approved-drug space, ChEMBL 37 max_phase=4 direct-interaction mechanisms (1,811 drugs, 650 human targets, 3,927 drug-gene rows), scored on three orthogonal lanes. Lane 1 network proximity: Guney z-scores against a pre-declared 12-gene MVA module over BioGRID 4.4.236 human physical PPI, 1,000 degree-matched nulls, seed 42 (calibrations: ivacaftor-CFTR z=-3.41, imatinib-BCR/ABL1 z=-10.66). Lane 2 knowledge graph: Bioteque disgenet-inferred bundle, cosine to the MVA1 node DOID:0080141 (self-edge AUC 0.917 calibration). Lane 3 signature reversal: BUB1B-knockdown proxy from GEO GSE92742 Phase I, 58 quality-gated signatures, tau-style connectivity over 205,034 compound signatures; the lane declares its own instrument limit (held-out-hairpin reconnection 0.101 vs null p95 0.184) and is used as weak evidence only. Structural allele tickets: RaSP stability scan on the AlphaFold model (N1002K ddG +2.41 kcal/mol in the validated I909T class; identity band +0.39 sd 0.58) and fpocket 4.2.3 (97 pockets, no druggable pocket at the locus). A pre-declared rule bans screen-score-only promotion; verdicts are graded on published direct evidence, regulator-verified status, and pediatric feasibility. Two further passes close gaps the lane screen left. First, the approved NAD+ precursors were graded by hand against the North 2014 NAD+/SIRT2-to-BubR1 mechanism, because niacin is an FDA-approved NAD+ precursor that the lane screen never scored: ChEMBL 37 holds no mechanism record for niacin or nicotinamide and a null-target record for acipimox, so target-annotated screening cannot see the class at all. Second, a bounded stabilizer computation asked whether any approved small molecule could act as a pharmacological chaperone on the pseudokinase domain: p2rank 2.4.2 (AlphaFold model) re-scanned pockets alongside fpocket, the nucleotide site was annotated by mapping the ADP contacts of the Drosophila crystal 6JKM onto human numbering (anchored at K795), and 2240 ligands were docked with smina against three boxes in two stages (35.5 CPU-hours), with ADP and ATP as references and a RaSP-derived stability-burden term per pocket.</t>
         </is>
       </c>
     </row>
@@ -703,7 +703,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Same discipline as v1 for literature and labels, and three extra manual checks for v2 claims: hydroxychloroquine and chloroquine pediatric label sections re-read on openFDA (including the &gt;=31 kg film-coated-tablet restriction), the FDA docket FDA-2023-P-0872 response of 2025-09-29 read directly for NMN status, and North 2014 (EMBO J; PMID 24825348) re-read to attribute the hypomorphic-cohort evidence to SIRT2 overexpression (not to NMN, which was given to wild-type mice).</t>
+          <t>Same discipline as v1 for literature and labels, and three extra manual checks for v2 claims: hydroxychloroquine and chloroquine pediatric label sections re-read on openFDA (including the &gt;=31 kg film-coated-tablet restriction), the FDA docket FDA-2023-P-0872 response of 2025-09-29 read directly for NMN status, and North 2014 (EMBO J; PMID 24825348) re-read to attribute the hypomorphic-cohort evidence to SIRT2 overexpression (not to NMN, which was given to wild-type mice). Regulator checks were extended to the NAD+ precursors: niacin's FDA applications and pediatric labeling were read from openFDA drug/drugsfda and drug/label, and acipimox's absence of any FDA application was confirmed the same way.</t>
         </is>
       </c>
     </row>
@@ -727,7 +727,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>ChEMBL 37 REST (mechanism/molecule/target). openFDA drug label records. BioGRID 4.4.236 tab3 human physical. Bioteque download API, disgenet bundle. GEO GSE92742 Level5 and metadata (sig_info, gene_info, pert_info). Ensembl REST (lookup, CDS map, sequence). UniProt O60566. AlphaFold DB AF-O60566-F1-model_v6. ClinVar VCV000533901.9, rs759242053. Europe PMC/PubMed for all mechanistic citations (PMID-tagged). EMA Translarna EPAR history (non-renewal 2025-03-28). FDA docket FDA-2023-P-0872 response of 2025-09-29 for NMN dietary-supplement status. RaSP code and model assets (MIT-licensed: Blaabjerg et al., eLife 2023) and fpocket 4.2.3 (Le Guilloux 2009).</t>
+          <t>ChEMBL 37 REST (mechanism/molecule/target). openFDA drug label records. BioGRID 4.4.236 tab3 human physical. Bioteque download API, disgenet bundle. GEO GSE92742 Level5 and metadata (sig_info, gene_info, pert_info). Ensembl REST (lookup, CDS map, sequence). UniProt O60566. AlphaFold DB AF-O60566-F1-model_v6. ClinVar VCV000533901.9, rs759242053. Europe PMC/PubMed for all mechanistic citations (PMID-tagged). EMA Translarna EPAR history (non-renewal 2025-03-28). FDA docket FDA-2023-P-0872 response of 2025-09-29 for NMN dietary-supplement status. RaSP code and model assets (MIT-licensed: Blaabjerg et al., eLife 2023) and fpocket 4.2.3 (Le Guilloux 2009). Additional sources for the v2 additions: RCSB PDB entries 6JKK and 6JKM plus UniProt A1Z6I7 for the cross-species ATP-site annotation, AlphaFold AF-O60566-F1-model_v6 as the docking receptor, p2rank 2.4.2, smina (AutoDock Vina 1.1.2 scoring), RDKit for ligand generation, and the ChEMBL approved-molecule structure set for the docking library.</t>
         </is>
       </c>
     </row>
@@ -751,7 +751,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Both alleles are loss of function, by different routes, all verified arithmetically. The stop-gain (c.2210T&gt;G, TTA to TGA UGA, tetranucleotide TGAA) sits in exon 17 of 23; recomputed live from Ensembl in v2, the PTC codon starts at CDS 2209 and the last exon-exon junction is at CDS 2957, a 748-nucleotide margin with six downstream junctions, far beyond the 50-nucleotide NMD rule, so the transcript is destroyed before translation. The context is permissive (UGA, TGAA), so NMD, not the context, blocks the readthrough class. The missense (c.3006T&gt;G, AAT to AAG) is a last-exon change escaping NMD; v2 quantifies it with RaSP at +2.41 kcal/mol, the validated mild-instability I909T class, and fpocket finds no druggable pocket at the locus. The disrupted pathway is the spindle assembly checkpoint; the consequence is constitutional mosaic variegated aneuploidy with predisposition to embryonal rhabdomyosarcoma, Wilms tumor, leukemia, and lymphoma.</t>
+          <t>Both alleles are loss of function, by different routes, all verified arithmetically. The stop-gain (c.2210T&gt;G, TTA to TGA UGA, tetranucleotide TGAA) sits in exon 17 of 23; recomputed live from Ensembl in v2, the PTC codon starts at CDS 2209 and the last exon-exon junction is at CDS 2957, a 748-nucleotide margin with six downstream junctions, far beyond the 50-nucleotide NMD rule, so the transcript is destroyed before translation. The context is permissive (UGA, TGAA), so NMD, not the context, blocks the readthrough class. The missense (c.3006T&gt;G, AAT to AAG) is a last-exon change escaping NMD; v2 quantifies it with RaSP at +2.41 kcal/mol, the validated mild-instability I909T class, and fpocket finds no druggable pocket at the locus. The disrupted pathway is the spindle assembly checkpoint; the consequence is constitutional mosaic variegated aneuploidy with predisposition to embryonal rhabdomyosarcoma, Wilms tumor, leukemia, and lymphoma. The pseudokinase domain was additionally probed for ligandability: two independent pocket finders agree there is no pocket at N1002 (nearest p2rank pocket 25.05 angstrom away; fpocket druggability at most 0.169 anywhere, 0.111 inside the domain, best p2rank probability 0.406), and no approved molecule stands out in docking against the nucleotide site, the N1002-adjacent pockets, or the domain's most druggable pocket.</t>
         </is>
       </c>
     </row>
@@ -763,7 +763,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>v1: about one analyst-day plus curation in a 36-hour window, CPU-only. v2: roughly one additional analyst-day on CPU-only infrastructure, including three bounded cluster jobs (the 23 GB LINCS board scan ~10 minutes, the 21,000-substitution RaSP scan, and the fpocket build/run) plus review.</t>
+          <t>v1: about one analyst-day plus curation in a 36-hour window, CPU-only. v2: roughly one additional analyst-day on CPU-only infrastructure, including three bounded cluster jobs (the 23 GB LINCS board scan ~10 minutes, the 21,000-substitution RaSP scan, and the fpocket build/run) plus review. The v2 additions added about 35.5 CPU-hours of docking plus minutes of pocket prediction, all CPU-only.</t>
         </is>
       </c>
     </row>
@@ -775,7 +775,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Track 2 v2 re-verifies the v1 mechanism chain and replaces qualitative class grading with a quantitative screen of the full approved-drug space. All 1,811 approved drugs with human protein targets in ChEMBL 37 were scored on three orthogonal lanes: network-proximity z-scores against a declared MVA module over the BioGRID human PPI with degree-matched nulls (calibrations pass: ivacaftor-CFTR z=-3.41, imatinib-BCR/ABL1 z=-10.66); knowledge-graph cosine to the MVA1 disease node DOID:0080141 in the Bioteque disgenet bundle (self-edge calibration AUC 0.917); and signature reversal over 205,034 LINCS Phase I compound signatures for a BUB1B-low proxy. The LINCS lane declares its instrument limit openly (hairpin discordance: held-out reconnection 0.101 vs null p95 0.184) and is downgraded to weak evidence that promotes nothing. Structural tickets close the product-locus picture: the nonsense transcript is NMD-destroyed (748-nucleotide margin, recomputed from Ensembl), and the missense allele reads as validated mild instability with no druggable pocket (RaSP +2.41 kcal/mol versus I909T +3.28 and L1012P +8.70; fpocket 97 pockets, none at the site). Under the pre-registered rule that screen scores alone never promote, no ingredient tops all three lanes, and the knowledge graph's loudest approved beat (fostamatinib, percentile 99.8) carries no published rescue-direction evidence or pediatric approval and is explicitly rejected. On direct published evidence the chloroquine/hydroxychloroquine class becomes the primary secondary-prevention hypothesis (Tang 2011 aneuploidy-selectivity; hydroxychloroquine's established pediatric malaria label, narrowed by the &gt;=31 kg tablet restriction), metformin is demoted to protection fallback for weak aneuploidy-selectivity support, NMN is graded the best biological but status-blocked dosage-raise route (lawful supplement since FDA's 2025-09-29 reversal, not an FDA-approved medication), and amlexanox stays bench-only. Strengths: quantifiability, calibrated lanes, pre-registered decision rule, recorded rejections. Limitations: the declared LINCS weakness, DisGeNET-inferred node bias, one-paper direction evidence for both promoted classes, and partial lane coverage (584 of 1,811 on the knowledge graph, 587 on LINCS). Bench falsification tests are named for the restore and protect chains.</t>
+          <t>Track 2 v2 re-verifies the v1 mechanism chain and replaces qualitative class grading with a quantitative screen of the full approved-drug space. All 1,811 approved drugs with human protein targets in ChEMBL 37 were scored on three orthogonal lanes: network-proximity z-scores against a declared MVA module over the BioGRID human PPI with degree-matched nulls (calibrations pass: ivacaftor-CFTR z=-3.41, imatinib-BCR/ABL1 z=-10.66); knowledge-graph cosine to the MVA1 disease node DOID:0080141 in the Bioteque disgenet bundle (self-edge calibration AUC 0.917); and signature reversal over 205,034 LINCS Phase I compound signatures for a BUB1B-low proxy. The LINCS lane declares its instrument limit openly (hairpin discordance: held-out reconnection 0.101 vs null p95 0.184) and is downgraded to weak evidence that promotes nothing. Structural tickets close the product-locus picture: the nonsense transcript is NMD-destroyed (748-nucleotide margin, recomputed from Ensembl), and the missense allele reads as validated mild instability with no druggable pocket (RaSP +2.41 kcal/mol versus I909T +3.28 and L1012P +8.70; fpocket 97 pockets, none at the site). Under the pre-registered rule that screen scores alone never promote, no ingredient tops all three lanes, and the knowledge graph's loudest approved beat (fostamatinib, percentile 99.8) carries no published rescue-direction evidence or pediatric approval and is explicitly rejected. On direct published evidence the chloroquine/hydroxychloroquine class becomes the primary secondary-prevention hypothesis (Tang 2011 aneuploidy-selectivity; hydroxychloroquine's established pediatric malaria label, narrowed by the &gt;=31 kg tablet restriction), metformin is demoted to protection fallback for weak aneuploidy-selectivity support, NMN is graded the best biological but status-blocked dosage-raise route (lawful supplement since FDA's 2025-09-29 reversal, not an FDA-approved medication), and amlexanox stays bench-only. Strengths: quantifiability, calibrated lanes, pre-registered decision rule, recorded rejections. Limitations: the declared LINCS weakness, DisGeNET-inferred node bias, one-paper direction evidence for both promoted classes, and partial lane coverage (584 of 1,811 on the knowledge graph, 587 on LINCS). Bench falsification tests are named for the restore and protect chains. Two additions complete the v2 picture. The NAD+ precursor class, which the target-annotated drug universe could not see (no ChEMBL mechanism record for niacin or nicotinamide, a null-target record for acipimox), was graded separately: niacin is an approved NAD+ precursor, so the dosage-raise axis is not empty of medicines, yet it is rejected for this case on evidence and pediatric labeling (safety and effectiveness not established in children; no BubR1 or aneuploidy data), while nicotinamide conflicts on direction through SIRT2 inhibition and acipimox has no FDA approval. A bounded stabilizer screen then tested the tafamidis-style possibility that a chaperone binds away from the mutation: after mapping the ADP site from the Drosophila crystal 6JKM onto human numbering (validated at K795), 2240 approved molecules were docked against three pockets in two stages (35.5 CPU-hours). The result is a negative bounded by a declared instrument limit: the engine could not reproduce the crystal ADP pose (6.03 angstrom), the natural nucleotides score no better than ordinary drugs, and no molecule separates from background, so a stabilizer route for this allele would require an experimentally discovered site rather than a repurposing hit.</t>
         </is>
       </c>
     </row>

</xml_diff>